<commit_message>
Label upcountry hubs as for consideration
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012MkqAAsvvPuHFRJJpDh8zC
</commit_message>
<xml_diff>
--- a/output/Makro_Darkstore_คัดเลือกฮับ.xlsx
+++ b/output/Makro_Darkstore_คัดเลือกฮับ.xlsx
@@ -1885,7 +1885,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>แนะนำเปิด</t>
+          <t>เพื่อใช้พิจารณา</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2718,6 +2718,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>

</xml_diff>